<commit_message>
refactor(player,data): move player values and item table to Luban
Task 5：Health.maxHealth 改由 Character 表解析（先解析再 ResetToFull）；PlayerMovement 的蹲/走/跑、重力、跳高、下落倍率、跳跃 CD、地面检测偏移、跌落阈值，PlayerController 的 Shift 长按阈值，PlayerLockOn 的锁定距离、PlayerAnimator 的锁定转向速度、PlayerDodge 的翻滚/位移/无敌帧/转身数值、ParrySystem 的弹反格挡数值全部改为读 Player/Parry 行；moveCurve 与动画相关字段仍在 Prefab。CharacterConfigIdentity 增加 GetCharacterRow/GetPlayerRow/GetStaminaRow/GetParryRow 统一解析入口。敌人提前接入 Character 表（enemy_default=1000），避免迁移中途 Play 被打断。Task 6：Item.txt 按 Tab 导入 Item Sheet（10001~10008 原 ID 与原值），DataRepository 改为从 Luban Item 行构建 DRItem 兼容视图并删除 ParseItemTable 死代码，Shop 仍走 TSV；校验器补 Player/Parry 行、Item asset_id 唯一性、Shop→Item 引用检查。batchmode 实测：8 items / 6 shop rows / 2 character / 1 player / 1 stamina / 1 parry，校验全部通过。
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/Gameplay.xlsx
+++ b/Config/Luban/Datas/Gameplay.xlsx
@@ -8,7 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stamina" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parry" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stamina" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,7 +460,6 @@
           <t>##group</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>c</t>
@@ -489,6 +491,16 @@
       </c>
       <c r="C5" t="n">
         <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>enemy_default</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1000</v>
       </c>
     </row>
   </sheetData>
@@ -502,6 +514,1378 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:W5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>##var</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>crouch_speed</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>walk_speed</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>run_speed</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>gravity</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>max_height</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>fall_multiplier</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>jump_cooldown</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>ground_check_offset</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>fall_height</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>run_hold_threshold</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>lock_on_distance</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>lock_on_turn_speed</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>dodge_duration</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>dodge_cooldown</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>dodge_distance</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>move_start_delay</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>move_duration</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>iframe_start_delay</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>iframe_duration</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>turn_to_dodge_dir_time</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>allow_neutral_dodge</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>##type</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>float#range=[0,50]</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>float#range=[0,50]</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>float#range=[0,50]</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>float#range=[-200,0]</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>float#range=[0,20]</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>float#range=[0,20]</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>float#range=[0,10]</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>float#range=[0,10]</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>float#range=[0,10]</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>float#range=[0,5]</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>float#range=[0,100]</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>float#range=[0,720]</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>float#range=[0,10]</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>float#range=[0,10]</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>float#range=[0,50]</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>float#range=[0,10]</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>float#range=[0,10]</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>float#range=[0,10]</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>float#range=[0,10]</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>float#range=[0,10]</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>##group</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>##</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>配置ID(引用Character.id)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>蹲下移动速度 m/s</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>行走速度 m/s</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>奔跑速度 m/s</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>重力加速度(负值)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>最大跳跃高度 m</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>下落加速度倍数</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>跳跃冷却(秒)</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>地面检测射线偏移 m</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>跌落判定阈值 m</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Shift 长按进入疾跑的阈值(秒)</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>锁定最大距离 m</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>锁定时转向速度(度/秒)</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>翻滚总时长(秒)</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>翻滚冷却(秒)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>翻滚位移距离 m</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>进入 Roll 后开始位移的等待(秒)</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>位移兜底时长(秒，读不到动画状态时用)</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>无敌帧起始延迟(秒，真实时间)</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>无敌帧持续(秒，真实时间)</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>非锁定翻滚转身时长(秒)</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>无方向输入时是否允许原地翻滚</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>player_main</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-9.800000000000001</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M5" t="n">
+        <v>15</v>
+      </c>
+      <c r="N5" t="n">
+        <v>8</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="W5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>##var</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>parry_window</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>enemy_stagger_duration</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>riposte_window</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>parry_invuln_duration</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>block_damage_reduction</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>block_still_knockback</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>##type</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>float#range=[0,10]</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>float#range=[0,30]</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>float#range=[0,30]</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>float#range=[0,10]</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>float#range=[0,1]</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>##group</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>##</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>配置ID(引用Character.id)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>按下格挡后仍算弹反成功的窗口(秒)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>弹反成功后敌人硬直(秒)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>弹反成功后玩家可反击窗口(秒)，0=不限制</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>弹反成功后短暂无敌(秒，真实时间)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>普通格挡减伤比例 0~1</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>格挡成功是否仍受击退</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>【未启用功能】当前工程没有 ParrySystem 实例与 ParryConfig 资产，本行只是开发初始值，不代表玩法已验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>player_main</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>##var</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>weapon_type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>base_damage</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>crit_rate</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>star</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>skill_description</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>image_path</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>asset_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>##type</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>int#range=[0,100000]</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>float#range=[0,1]</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>int#range=[0,100]</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>##group</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>##</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>物品ID（保持原值，不得重新编号）</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>物品类型(1武器/2食物/3盾)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>武器类型(E_WeaponType 整数，非武器填 -1)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>基础伤害</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>暴击率 0~1</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>星级</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>技能描述</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>图标 Resources 路径</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>资源ID（非空且唯一）</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="n">
+        <v>10001</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Sever</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Sealed under ice for millennia. This ancient blade contains the power of eternal frost.</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Using [Sever - Moment of Extreme Cold] freezes time itself. Allows the wielder to strike before fate unfolds.</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Sprites/UI/Weapon/weapon_01</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Item_Sever</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="n">
+        <v>10002</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Demon Breaker</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Emitting a chilling demonic aura. This blade was forged in the abyss to hunt the unholy.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Use [Demon Breaker] to fire countless projectiles that pierce through all enemies in their path.</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Sprites/UI/Weapon/weapon_02</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Item_DemonBreaker</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="n">
+        <v>10003</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>14</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Ascending Dragon</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>A spear nurtured above thunderclouds. Crackling with the fury of a thousand storms.</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Use [Thunder Shock] to summon thunderclouds that unleash automatic lightning strikes upon foes.</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Sprites/UI/Weapon/weapon_04</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Item_AscendingDragon</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="n">
+        <v>10004</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>10</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Hunting Bow</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>A sturdy longbow carved from ancient oak. Favored by rangers of the northern valleys.</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Use [Thunderclap] to call down a single devastating bolt from the heavens.</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Sprites/UI/Weapon/weapon_08</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Item_HuntingBow</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="n">
+        <v>10005</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Sandwich</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>GoodFood</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Eating it!</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Sprites/UI/Food/Food02</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Item_Sandwich</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="n">
+        <v>10006</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Salmon caviar</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Good!Good!Good!</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Up!</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Sprites/UI/Food/Food03</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Item_Salmon caviar</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="n">
+        <v>10007</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>13</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Axe</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>SharpAxe��</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>OhYes!</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Sprites/UI/Weapon/weapon_03</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Item_Axe</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="n">
+        <v>10008</v>
+      </c>
+      <c r="C12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Round Shield</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>A sturdy round shield forged for the frontline.</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Raise it to block incoming strikes.</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Sprites/UI/Weapon/weapon_05</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Item_RoundShield</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
refactor(weapon): move weapon and upgrade values to Luban
Weapon 表（map，主键 weapon_id）+ WeaponUpgrade 表（one）：WeaponConfig 的攻击距离/弹药/冷却/弹速/散布改为按 weaponID 读表，属性名保持原拼写（含 projectilleSpeed），RangedFighter 无需改动；WeaponUpgradeSystem 的等级上限/伤害/暴击/费用系数改为读单行表，公式与整数返回不变。四个 WeaponConfig 资产已重存，YAML 里已迁移数值与历史孤立字段（weaponType/baseDamage）一并清除，模型/动画/招式引用未动。校验器新增：weaponID 非空/不重复/有 Weapon 行、Weapon.weapon_id→Item.id、Weapon 行必须有对应 SO，并把弓 1111 的既有缺陷作为【已知缺陷】单列（不计失败，按用户决定本次不修）。batchmode 实测校验通过。
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/Gameplay.xlsx
+++ b/Config/Luban/Datas/Gameplay.xlsx
@@ -12,6 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parry" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stamina" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weapon" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeaponUpgrade" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1401,7 +1403,6 @@
           <t>##group</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>c</t>
@@ -2195,4 +2196,406 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>##var</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>weapon_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>attack_range</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>max_ammo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>fire_cooldown</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>projectile_speed</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>aim_spread_angle</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>hip_fire_spread_angle</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>##type</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>float#range=[0,100]</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>int#range=[0,9999]</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>float#range=[0,60]</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>float#range=[0,1000]</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>float#range=[0,180]</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>float#range=[0,180]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>##group</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>##</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>主键=WeaponConfig.weaponID，正常应对应 Item.id</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>攻击距离（米）。当前工程没有消费方，仅数据等价</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>最大弹药量</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>射击冷却（秒）</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>投射物速度（米/秒）</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>瞄准散布角度（度）</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>腰射散布角度（度）</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="n">
+        <v>10001</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>30</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>25</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="n">
+        <v>10007</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>25</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="n">
+        <v>10008</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>30</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F7" t="n">
+        <v>25</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="n">
+        <v>1111</v>
+      </c>
+      <c r="C8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>30</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>25</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>##var</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>max_level</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>damage_per_level</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>crit_rate_per_level</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>upgrade_cost_per_level</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>##type</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>int#range=[1,9999]</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>int#range=[0,1000]</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>float#range=[0,10]</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>int#range=[0,10000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>##group</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>##</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>武器最高等级</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>每级增加的基础伤害</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>每级增加的暴击率</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>升级费用公式中的系数：cost = (当前等级 + 1) × 本值</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="n">
+        <v>90</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="E5" t="n">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
refactor(combat): move attack tuning values to Luban
Attack 表（map，主键 attack_id）：命中窗口/伤害倍率/削韧/可弹反/卡肉时长与缩放改为按 attackId 读表，AttackData 只保留 AnimName、HitboxToUse 与新增的稳定 attackId。9 个 AttackData 资产已写入 attackId（= 当前资产名）并清除 YAML 中的旧数值。校验器新增：attackId 非空/不重复/有 Attack 行、命中窗口 start<=end、Attack 行必须有对应资产。batchmode 实测校验通过。
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/Gameplay.xlsx
+++ b/Config/Luban/Datas/Gameplay.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stamina" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weapon" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeaponUpgrade" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attack" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2297,7 +2298,6 @@
           <t>##group</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>c</t>
@@ -2537,7 +2537,6 @@
           <t>##group</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>c</t>
@@ -2593,6 +2592,461 @@
       </c>
       <c r="E5" t="n">
         <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>##var</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>attack_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>impact_start_time</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>impact_end_time</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>damage_multiplier</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>poise_damage</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>parryable</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>hit_stop_duration</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>hit_stop_time_scale</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>##type</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>float#range=[0,5]</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>float#range=[0,5]</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>float#range=[0,100]</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>float#range=[0,1000]</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>float#range=[-1,10]</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>float#range=[-1,1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>##group</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>##</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>稳定招式ID（首次填表用资产名，之后不再随资产改名）</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>命中窗口起点（动画归一化时间）</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>命中窗口终点（必须 &gt;= 起点）</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>伤害倍率（相对武器基础伤害）</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>削韧值（当前无消费方）</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>是否可被弹反</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>卡肉时长（秒）；&lt;0 用 HitStopManager 默认值</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>卡肉时间缩放；有效范围 0~1，&lt;0 用默认值</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Sword_Attack1</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Sword_Attack2</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Sword_Attack3</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>10</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Axe_Attack1</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>10</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Axe_Attack2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Axe_Attack3</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Slash</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>10</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>OutwardSlash</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>10</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Kick</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>10</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor(combat): externalize global damage and hit-stop values
新增 CombatGlobal 单行表：DamageRouter.FallbackBaseDamage 由常量改为读表（只在武器 ID 解析失败时使用），HitStopManager 的默认卡肉时长/时间缩放/上限改为读表并在 Awake 解析一次；Time.timeScale 所有权与暂停优先逻辑不变。校验器新增单行表取值范围检查。batchmode 实测校验通过。
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/Gameplay.xlsx
+++ b/Config/Luban/Datas/Gameplay.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weapon" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeaponUpgrade" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attack" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatGlobal" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2708,6 +2709,420 @@
           <t>##group</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>##</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>稳定招式ID（首次填表用资产名，之后不再随资产改名）</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>命中窗口起点（动画归一化时间）</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>命中窗口终点（必须 &gt;= 起点）</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>伤害倍率（相对武器基础伤害）</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>削韧值（当前无消费方）</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>是否可被弹反</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>卡肉时长（秒）；&lt;0 用 HitStopManager 默认值</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>卡肉时间缩放；有效范围 0~1，&lt;0 用默认值</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Sword_Attack1</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Sword_Attack2</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Sword_Attack3</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>10</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Axe_Attack1</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>10</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Axe_Attack2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Axe_Attack3</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Slash</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>10</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>OutwardSlash</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>10</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Kick</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>10</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>##var</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>fallback_base_damage</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>default_hit_stop_duration</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>default_hit_stop_time_scale</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>max_hit_stop_duration</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>##type</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>float#range=[0,10000]</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>float#range=[0,5]</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>float#range=[0,1]</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>float#range=[0,5]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>##group</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
@@ -2729,26 +3144,6 @@
           <t>c</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2758,295 +3153,37 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>稳定招式ID（首次填表用资产名，之后不再随资产改名）</t>
+          <t>武器ID解析失败时的兜底基础伤害</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>命中窗口起点（动画归一化时间）</t>
+          <t>默认卡肉时长（秒，真实时间）</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>命中窗口终点（必须 &gt;= 起点）</t>
+          <t>默认卡肉时间缩放 0~1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>伤害倍率（相对武器基础伤害）</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>削韧值（当前无消费方）</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>是否可被弹反</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>卡肉时长（秒）；&lt;0 用 HitStopManager 默认值</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>卡肉时间缩放；有效范围 0~1，&lt;0 用默认值</t>
+          <t>单次卡肉时长上限（秒）</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Sword_Attack1</t>
-        </is>
+      <c r="B5" t="n">
+        <v>5</v>
       </c>
       <c r="C5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E5" t="n">
         <v>0.3</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="E5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" t="n">
-        <v>10</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Sword_Attack2</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="E6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" t="n">
-        <v>10</v>
-      </c>
-      <c r="G6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Sword_Attack3</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="E7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" t="n">
-        <v>10</v>
-      </c>
-      <c r="G7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Axe_Attack1</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="E8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" t="n">
-        <v>10</v>
-      </c>
-      <c r="G8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Axe_Attack2</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="E9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" t="n">
-        <v>10</v>
-      </c>
-      <c r="G9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Axe_Attack3</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" t="n">
-        <v>10</v>
-      </c>
-      <c r="G10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="n">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Slash</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" t="n">
-        <v>10</v>
-      </c>
-      <c r="G11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" t="n">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>OutwardSlash</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="E12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" t="n">
-        <v>10</v>
-      </c>
-      <c r="G12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" t="n">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Kick</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="E13" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" t="n">
-        <v>10</v>
-      </c>
-      <c r="G13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" t="n">
-        <v>-1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor(enemy): move controller and FSM tuning to Luban
新增 Enemy 表（map，主键 id=Character.id，25 个字段）：EnemyController 的 fov/警戒范围/最小间距/分离力/演出锁超时，以及巡逻、攻击、环绕、后撤、受击、死亡各 FSM 状态的数值全部改为读该行（原来硬编码的 3.5 巡逻后速度、0.3 起手容差、500 后撤转身速度也一并入表）。EnemyController 在 Awake 解析一次并通过 Config 暴露只读入口，各状态不再各自持有序列化数值。Enemy.prefab 上已迁移的 19 行数值被清除。校验器新增：带 EnemyController 的 Prefab 必须有 Enemy 行、Enemy 行必须对上 Character 行、时间区间与 FOV 范围检查。batchmode 实测校验通过。
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/Gameplay.xlsx
+++ b/Config/Luban/Datas/Gameplay.xlsx
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeaponUpgrade" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attack" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatGlobal" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemy" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -512,6 +513,623 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>##var</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>fov</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>alert_range</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>min_separation_distance</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>separation_force</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>performance_lock_timeout</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>patrol_speed</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>patrol_forward_anim_speed</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>arrival_distance</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>combat_nav_speed</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>attack_distance</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>attack_distance_tolerance</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>circling_speed</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>distance_to_sand</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>adjust_distance_threshold</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>idle_time_min</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>idle_time_max</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>circling_time_min</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>circling_time_max</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>keep_attacking_dead_target_seconds</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>backward_walk_speed</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>distance_to_retreat</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>retreat_turn_speed</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>stun_time</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>destroy_delay</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>##type</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>float#range=[0,360]</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>float#range=[0,200]</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>float#range=[0,20]</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>float#range=[0,200]</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>float#range=[0,120]</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>float#range=[0,50]</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>float#range=[0,50]</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>float#range=[0,20]</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>float#range=[0,50]</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>float#range=[0,50]</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>float#range=[0,20]</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>float#range=[0,360]</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>float#range=[0,50]</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>float#range=[0,50]</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>float#range=[0,60]</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>float#range=[0,60]</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>float#range=[0,60]</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>float#range=[0,60]</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>float#range=[0,600]</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>float#range=[0,50]</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>float#range=[0,50]</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>float#range=[0,3600]</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>float#range=[0,60]</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>float#range=[0,300]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>##group</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>##</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>配置ID(引用Character.id)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>视野角度(度)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>警戒范围(米)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>与玩家保持的最小间距(米)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>分离推力强度</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>配对演出锁最长持续(秒)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>巡逻移动速度</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>巡逻时 forwardSpeed 动画参数</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>到达路径点判定距离(米)</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>巡逻结束后的 NavMeshAgent 速度(原硬编码 3.5)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>发动攻击的距离(米)</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>攻击起手额外容差(米，原硬编码 0.3)</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>环绕转向速度(度/秒)</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>战斗站立距离(米)</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>距离修正阈值(米)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>待机时间下限(秒)</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>待机时间上限(秒)</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>环绕时间下限(秒)</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>环绕时间上限(秒)</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>目标倒地后继续补刀的秒数</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>后撤速度</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>后撤距离(米)</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>后撤转身速度(度/秒，原硬编码 500)</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>受击硬直(秒)</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>尸体销毁延迟(秒)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>enemy_default</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>180</v>
+      </c>
+      <c r="D5" t="n">
+        <v>20</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K5" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="N5" t="n">
+        <v>20</v>
+      </c>
+      <c r="O5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>2</v>
+      </c>
+      <c r="R5" t="n">
+        <v>5</v>
+      </c>
+      <c r="S5" t="n">
+        <v>3</v>
+      </c>
+      <c r="T5" t="n">
+        <v>6</v>
+      </c>
+      <c r="U5" t="n">
+        <v>4</v>
+      </c>
+      <c r="V5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="W5" t="n">
+        <v>3</v>
+      </c>
+      <c r="X5" t="n">
+        <v>500</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -3123,7 +3741,6 @@
           <t>##group</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>c</t>

</xml_diff>

<commit_message>
refactor(enemy): externalize global attack scheduling values
新增 EnemyGlobal 单行表：EnemyManager 的出手间隔区间（原 Vector2）、初始出手倒计时、非锁定最近目标刷新周期改为读表；运行时倒计时仍是组件状态，不回写表格。EnemyManager.prefab 重存后清掉 timeRangeBetWeenAttacks。校验器新增单行表区间/非负/刷新周期检查。batchmode 实测校验通过。
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/Gameplay.xlsx
+++ b/Config/Luban/Datas/Gameplay.xlsx
@@ -17,6 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attack" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatGlobal" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemy" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyGlobal" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -792,6 +793,412 @@
           <t>##group</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>##</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>配置ID(引用Character.id)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>视野角度(度)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>警戒范围(米)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>与玩家保持的最小间距(米)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>分离推力强度</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>配对演出锁最长持续(秒)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>巡逻移动速度</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>巡逻时 forwardSpeed 动画参数</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>到达路径点判定距离(米)</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>巡逻结束后的 NavMeshAgent 速度(原硬编码 3.5)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>发动攻击的距离(米)</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>攻击起手额外容差(米，原硬编码 0.3)</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>环绕转向速度(度/秒)</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>战斗站立距离(米)</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>距离修正阈值(米)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>待机时间下限(秒)</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>待机时间上限(秒)</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>环绕时间下限(秒)</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>环绕时间上限(秒)</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>目标倒地后继续补刀的秒数</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>后撤速度</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>后撤距离(米)</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>后撤转身速度(度/秒，原硬编码 500)</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>受击硬直(秒)</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>尸体销毁延迟(秒)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>enemy_default</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>180</v>
+      </c>
+      <c r="D5" t="n">
+        <v>20</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K5" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="N5" t="n">
+        <v>20</v>
+      </c>
+      <c r="O5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>2</v>
+      </c>
+      <c r="R5" t="n">
+        <v>5</v>
+      </c>
+      <c r="S5" t="n">
+        <v>3</v>
+      </c>
+      <c r="T5" t="n">
+        <v>6</v>
+      </c>
+      <c r="U5" t="n">
+        <v>4</v>
+      </c>
+      <c r="V5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="W5" t="n">
+        <v>3</v>
+      </c>
+      <c r="X5" t="n">
+        <v>500</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>##var</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>attack_interval_min</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>attack_interval_max</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>initial_attack_delay</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>target_refresh_interval</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>##type</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>float#range=[0,600]</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>float#range=[0,600]</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>float#range=[0,600]</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>float#range=[0.001,10]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>##group</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
@@ -813,106 +1220,6 @@
           <t>c</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -922,207 +1229,37 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>配置ID(引用Character.id)</t>
+          <t>连续出手最小间隔(秒)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>视野角度(度)</t>
+          <t>连续出手最大间隔(秒)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>警戒范围(米)</t>
+          <t>敌人管理器初始出手倒计时(秒)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>与玩家保持的最小间距(米)</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>分离推力强度</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>配对演出锁最长持续(秒)</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>巡逻移动速度</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>巡逻时 forwardSpeed 动画参数</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>到达路径点判定距离(米)</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>巡逻结束后的 NavMeshAgent 速度(原硬编码 3.5)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>发动攻击的距离(米)</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>攻击起手额外容差(米，原硬编码 0.3)</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>环绕转向速度(度/秒)</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>战斗站立距离(米)</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>距离修正阈值(米)</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>待机时间下限(秒)</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>待机时间上限(秒)</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>环绕时间下限(秒)</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>环绕时间上限(秒)</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>目标倒地后继续补刀的秒数</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>后撤速度</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>后撤距离(米)</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>后撤转身速度(度/秒，原硬编码 500)</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>受击硬直(秒)</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>尸体销毁延迟(秒)</t>
+          <t>非锁定时最近目标刷新周期(秒)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>enemy_default</t>
-        </is>
+      <c r="B5" t="n">
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="F5" t="n">
-        <v>5</v>
-      </c>
-      <c r="G5" t="n">
-        <v>10</v>
-      </c>
-      <c r="H5" t="n">
-        <v>2</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K5" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="L5" t="n">
-        <v>1</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="N5" t="n">
-        <v>20</v>
-      </c>
-      <c r="O5" t="n">
-        <v>3</v>
-      </c>
-      <c r="P5" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>2</v>
-      </c>
-      <c r="R5" t="n">
-        <v>5</v>
-      </c>
-      <c r="S5" t="n">
-        <v>3</v>
-      </c>
-      <c r="T5" t="n">
-        <v>6</v>
-      </c>
-      <c r="U5" t="n">
-        <v>4</v>
-      </c>
-      <c r="V5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="W5" t="n">
-        <v>3</v>
-      </c>
-      <c r="X5" t="n">
-        <v>500</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>4</v>
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor(boss): move phase thresholds to Luban
新增 BossPhase 表（list，联合主键 boss_id+phase_index）。当前工程没有 Boss 实例也没有 BossPhaseConfig 资产，因此表【故意为空】，只建立表结构、生成代码与读取链路，不虚构 Boss 数据。DataRepository.GetBossPhases 按 boss_id 分组并按 phase_index 升序缓存；BossPhaseController 改为查询该列表，保留原有「反向遍历 + 只发一次阶段事件」的行为与 bossId 事件参数。校验器新增联合主键唯一、阈值 0~1、同 Boss 内严格递减检查。Boss Play 验证【未覆盖】。
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/Gameplay.xlsx
+++ b/Config/Luban/Datas/Gameplay.xlsx
@@ -18,6 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatGlobal" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemy" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyGlobal" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhase" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1199,7 +1200,6 @@
           <t>##group</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>c</t>
@@ -1260,6 +1260,109 @@
       </c>
       <c r="E5" t="n">
         <v>0.1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>##var</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>boss_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>phase_index</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>health_threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>##type</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>int#range=[0,99]</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>float#range=[0,1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>##group</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>##</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Boss 配置/事件标识</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>阶段序号（同一 Boss 内唯一，从 0 开始）</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>进入该阶段的血量比例阈值 0~1（同一 Boss 内不得重复）</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(config): align the bow weapon id with its item row
弓原来装备不上：BowConfig.weaponID = 1111，而 WeaponManager 的查找表以 weaponID 为键、
装备时用 item.id 去查，Item 表里对应的是 10004 Hunting Bow → TryGetValue 必然失败，
EquipWeapon 直接 return false。同时 Item 10004 的 weapon_type 被标成 Dagger(1)，
会让 MovesetResolver.IsMeleeWeapon 把弓当近战武器。

改动（按 Config/README.md §5 记录过的修复流程做）：
- Gameplay.xlsx：Weapon 表 1111 行改为 10004；Item 表 10004 的 weapon_type 改为 3(Bow)。
  重新执行 Luban 导出（gen_gameplay_json.bat，--strict 通过），只有 item.json / weapon.json 变化，
  生成的 C# 无 diff。
- BowConfig.weaponID 改为 10004。物品类型改成 Bow 后右槽 allowedTypes {0,1,2,3} 仍然接受，
  装备不会因为类型被拒。
- ConfigReferenceValidator：删掉按 1111 判定的「已知缺陷」分支，改回普通错误；
  Problem.IsKnownIssue 机制保留（当前没有登记项）。
- Config/README.md §5 与 CLAUDE.md「已知边界」改为已修复状态，并记下遗留：
  BowConfig.animOverride 指向玩家的基础控制器（类型不匹配 → 运行时为 null），弓没有专属动作覆盖。

验证：Assembly-CSharp / Assembly-CSharp-Editor 均 0 错误。
Play 验证：背包里装备 Hunting Bow → 右键进右肩 → 左键发射
（冷却 0.5s / 弹速 25 / 瞄射散布 1° 来自 Weapon 表 10004 行）。
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/Gameplay.xlsx
+++ b/Config/Luban/Datas/Gameplay.xlsx
@@ -2659,7 +2659,7 @@
         <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E8" t="n">
         <v>10</v>
@@ -3441,7 +3441,7 @@
     </row>
     <row r="8">
       <c r="B8" t="n">
-        <v>1111</v>
+        <v>10004</v>
       </c>
       <c r="C8" t="n">
         <v>5</v>

</xml_diff>